<commit_message>
Milestone: 2nd stage chats with client and satisfied.
</commit_message>
<xml_diff>
--- a/Copy of 自营司机运力表.xlsx
+++ b/Copy of 自营司机运力表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\派单\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E76AEC8-59F2-4836-94AC-2B94FDC3577F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482D9DAA-153B-40DD-8345-6CCB6C06FF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,9 +79,6 @@
     <t>白班</t>
   </si>
   <si>
-    <t>浦机</t>
-  </si>
-  <si>
     <t>早5晚18之前</t>
   </si>
   <si>
@@ -326,6 +323,9 @@
   </si>
   <si>
     <t>时间</t>
+  </si>
+  <si>
+    <t>浦东机场</t>
   </si>
 </sst>
 </file>
@@ -954,7 +954,7 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>1</v>
@@ -969,7 +969,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1">
@@ -992,16 +992,16 @@
         <v>8</v>
       </c>
       <c r="G2" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="I2" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="3" customFormat="1">
@@ -1009,13 +1009,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="D3" s="13" t="s">
         <v>17</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>18</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>12</v>
@@ -1024,16 +1024,16 @@
         <v>8</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1041,13 +1041,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="13" t="s">
         <v>21</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>22</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>12</v>
@@ -1056,16 +1056,16 @@
         <v>8</v>
       </c>
       <c r="G4" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="I4" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:13" s="4" customFormat="1">
@@ -1073,31 +1073,31 @@
         <v>4</v>
       </c>
       <c r="B5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="E5" s="17" t="s">
         <v>25</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>26</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I5" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1105,13 +1105,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="D6" s="13" t="s">
         <v>29</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>30</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>12</v>
@@ -1120,16 +1120,16 @@
         <v>8</v>
       </c>
       <c r="G6" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="I6" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1137,31 +1137,31 @@
         <v>6</v>
       </c>
       <c r="B7" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>33</v>
-      </c>
       <c r="E7" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1169,10 +1169,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>35</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>36</v>
       </c>
       <c r="D8" s="19">
         <v>18048018178</v>
@@ -1181,19 +1181,19 @@
         <v>12</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K8" s="18"/>
       <c r="L8" s="21"/>
@@ -1203,10 +1203,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>38</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>39</v>
       </c>
       <c r="D9" s="21">
         <v>13603700333</v>
@@ -1215,19 +1215,19 @@
         <v>12</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K9" s="18"/>
       <c r="L9" s="21"/>
@@ -1237,31 +1237,31 @@
         <v>9</v>
       </c>
       <c r="B10" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="D10" s="21" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>43</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:13" s="5" customFormat="1">
@@ -1280,31 +1280,31 @@
         <v>1</v>
       </c>
       <c r="B12" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="D12" s="29" t="s">
         <v>47</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>48</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I12" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:13" s="1" customFormat="1">
@@ -1312,31 +1312,31 @@
         <v>2</v>
       </c>
       <c r="B13" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="D13" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="31" t="s">
-        <v>52</v>
-      </c>
       <c r="E13" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="I13" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1344,31 +1344,31 @@
         <v>3</v>
       </c>
       <c r="B14" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="D14" s="33" t="s">
         <v>54</v>
-      </c>
-      <c r="D14" s="33" t="s">
-        <v>55</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="6" customFormat="1">
@@ -1376,31 +1376,31 @@
         <v>4</v>
       </c>
       <c r="B15" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="D15" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="35" t="s">
+      <c r="E15" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="F15" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="I15" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>
@@ -1411,31 +1411,31 @@
         <v>5</v>
       </c>
       <c r="B16" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="37" t="s">
         <v>61</v>
-      </c>
-      <c r="C16" s="37" t="s">
-        <v>62</v>
       </c>
       <c r="D16" s="38">
         <v>15001814303</v>
       </c>
       <c r="E16" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="H16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F16" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="I16" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:14" s="4" customFormat="1">
@@ -1443,31 +1443,31 @@
         <v>6</v>
       </c>
       <c r="B17" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="D17" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="D17" s="39" t="s">
-        <v>66</v>
-      </c>
       <c r="E17" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G17" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="I17" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K17" s="40"/>
       <c r="L17" s="41"/>
@@ -1477,31 +1477,31 @@
         <v>7</v>
       </c>
       <c r="B18" s="42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="C18" s="43" t="s">
+      <c r="D18" s="44" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="44" t="s">
+      <c r="E18" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="H18" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F18" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="G18" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="I18" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J18" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K18" s="18"/>
       <c r="L18" s="18"/>
@@ -1511,31 +1511,31 @@
         <v>8</v>
       </c>
       <c r="B19" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="45" t="s">
+      <c r="D19" s="46" t="s">
         <v>72</v>
-      </c>
-      <c r="D19" s="46" t="s">
-        <v>73</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:14" s="4" customFormat="1">
@@ -1543,31 +1543,31 @@
         <v>9</v>
       </c>
       <c r="B20" s="47" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="C20" s="47" t="s">
+      <c r="D20" s="47" t="s">
         <v>76</v>
       </c>
-      <c r="D20" s="47" t="s">
-        <v>77</v>
-      </c>
       <c r="E20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F20" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="I20" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K20" s="18"/>
       <c r="L20" s="18"/>
@@ -1577,31 +1577,31 @@
         <v>10</v>
       </c>
       <c r="B21" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="D21" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="48" t="s">
-        <v>80</v>
-      </c>
       <c r="E21" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H21" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F21" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="I21" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:14" s="1" customFormat="1">
@@ -1609,31 +1609,31 @@
         <v>11</v>
       </c>
       <c r="B22" s="49" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="49" t="s">
+      <c r="D22" s="49" t="s">
         <v>82</v>
-      </c>
-      <c r="D22" s="49" t="s">
-        <v>83</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G22" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H22" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="I22" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:14" s="1" customFormat="1">
@@ -1641,31 +1641,31 @@
         <v>12</v>
       </c>
       <c r="B23" s="50" t="s">
+        <v>83</v>
+      </c>
+      <c r="C23" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="D23" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="D23" s="51" t="s">
-        <v>86</v>
-      </c>
       <c r="E23" s="52" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F23" s="52" t="s">
-        <v>45</v>
-      </c>
-      <c r="G23" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="I23" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:14" s="1" customFormat="1">
@@ -1673,31 +1673,31 @@
         <v>13</v>
       </c>
       <c r="B24" s="53" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="53" t="s">
         <v>87</v>
       </c>
-      <c r="C24" s="53" t="s">
+      <c r="D24" s="53" t="s">
         <v>88</v>
-      </c>
-      <c r="D24" s="53" t="s">
-        <v>89</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K24" s="18"/>
       <c r="L24" s="18"/>

</xml_diff>

<commit_message>
Implementation on the 3rd milestone with more experiment and bug fixing
</commit_message>
<xml_diff>
--- a/Copy of 自营司机运力表.xlsx
+++ b/Copy of 自营司机运力表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\派单\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482D9DAA-153B-40DD-8345-6CCB6C06FF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2411E054-8980-48EE-8F92-46AF66641765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11940" yWindow="765" windowWidth="15795" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -935,6 +935,8 @@
   <dimension ref="A1:N24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.7109375" customWidth="1"/>
     <col min="8" max="8" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>

</xml_diff>